<commit_message>
Apply declared Replus cover color links and final dimension flow
</commit_message>
<xml_diff>
--- a/changes/replus-runtime-v5/candidates/RPL_ATT_TH.xlsx
+++ b/changes/replus-runtime-v5/candidates/RPL_ATT_TH.xlsx
@@ -1,46 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90_Evidence" sheetId="1" r:id="R2b6e6ed7bada442f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_INDEX" sheetId="2" r:id="R4dd48d2db36d46c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_README" sheetId="3" r:id="R1c1dea0e288d4d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_入力フロー" sheetId="4" r:id="R272ff3e1e3534a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_取替方式" sheetId="5" r:id="R2f83c62ea1904f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02A_仕様区分" sheetId="6" r:id="R5e733d38c08b42fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_窓種" sheetId="7" r:id="R69b3d3c4b9504f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03A_枠仕様" sheetId="8" r:id="R5a090c82d70a42cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03B_窓種枠設定" sheetId="9" r:id="Rcfa3a0a0edd147b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_窓種固有仕様" sheetId="10" r:id="Ra9a4974142d64386"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_サイズルール" sheetId="11" r:id="R985f115631254d86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05A_サイズ区間" sheetId="12" r:id="R83f6f4860db1464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05B_境界ルール" sheetId="13" r:id="R56cd6145e3c04c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_色" sheetId="14" r:id="R0288233248c84f1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06A_色適用条件" sheetId="15" r:id="Re12bb10f737d40dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_網戸" sheetId="16" r:id="R3444f7a787604510"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07A_網戸適用条件" sheetId="17" r:id="R5651d1f3491145de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ガラス" sheetId="18" r:id="R35456ba997884500"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08A_ガラス適用条件" sheetId="19" r:id="Rb944e66ab8b043c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_その他OP" sheetId="20" r:id="Reaac98e3de13430a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09A_OP依存関係" sheetId="21" r:id="Re81979da90f9481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_適用条件" sheetId="22" r:id="Rbcb5d791d6614268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10A_既設窓互換" sheetId="23" r:id="R78119a376b004a3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10B_現調項目" sheetId="24" r:id="R7d00c7b2c75c4c05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99_QA" sheetId="25" r:id="Raac614bf84584871"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04A_開口構成" sheetId="26" r:id="R874b6fc902ca49ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_見積入力テスト" sheetId="27" r:id="Re299fc62d7274adb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10C_化粧カバー見付" sheetId="28" r:id="R37f3a0b9ef08489f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02B_参照商品" sheetId="29" r:id="R2c486cecd873439e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02C_新設サッシ手配方式" sheetId="30" r:id="Rd1eb13f484ca4237"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03C_対応サーモス窓種" sheetId="31" r:id="Rae90d07059364f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03D_サーモス参照制限" sheetId="32" r:id="R096c7adca96149e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05C_寸法変換" sheetId="33" r:id="R525f69380852497b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_共通参照" sheetId="34" r:id="R7af534a981d14c8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02D_対応シリーズ" sheetId="35" r:id="R0774209512b74aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12A_ATT_TW比較" sheetId="36" r:id="R3603ed6ba51543df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_参照整合性監査" sheetId="37" r:id="R42ed65090b1d4ecf"/>
-  </x:sheets>
-</x:workbook>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="90_Evidence" sheetId="1" r:id="R2b6e6ed7bada442f"/>
+    <sheet name="00_INDEX" sheetId="2" r:id="R4dd48d2db36d46c8"/>
+    <sheet name="00_README" sheetId="3" r:id="R1c1dea0e288d4d4c"/>
+    <sheet name="01_入力フロー" sheetId="4" r:id="R272ff3e1e3534a7d"/>
+    <sheet name="02_取替方式" sheetId="5" r:id="R2f83c62ea1904f4d"/>
+    <sheet name="02A_仕様区分" sheetId="6" r:id="R5e733d38c08b42fd"/>
+    <sheet name="03_窓種" sheetId="7" r:id="R69b3d3c4b9504f57"/>
+    <sheet name="03A_枠仕様" sheetId="8" r:id="R5a090c82d70a42cd"/>
+    <sheet name="03B_窓種枠設定" sheetId="9" r:id="Rcfa3a0a0edd147b9"/>
+    <sheet name="04_窓種固有仕様" sheetId="10" r:id="Ra9a4974142d64386"/>
+    <sheet name="05_サイズルール" sheetId="11" r:id="R985f115631254d86"/>
+    <sheet name="05A_サイズ区間" sheetId="12" r:id="R83f6f4860db1464c"/>
+    <sheet name="05B_境界ルール" sheetId="13" r:id="R56cd6145e3c04c44"/>
+    <sheet name="06_色" sheetId="14" r:id="R0288233248c84f1e"/>
+    <sheet name="06A_色適用条件" sheetId="15" r:id="Re12bb10f737d40dd"/>
+    <sheet name="07_網戸" sheetId="16" r:id="R3444f7a787604510"/>
+    <sheet name="07A_網戸適用条件" sheetId="17" r:id="R5651d1f3491145de"/>
+    <sheet name="08_ガラス" sheetId="18" r:id="R35456ba997884500"/>
+    <sheet name="08A_ガラス適用条件" sheetId="19" r:id="Rb944e66ab8b043c3"/>
+    <sheet name="09_その他OP" sheetId="20" r:id="Reaac98e3de13430a"/>
+    <sheet name="09A_OP依存関係" sheetId="21" r:id="Re81979da90f9481f"/>
+    <sheet name="10_適用条件" sheetId="22" r:id="Rbcb5d791d6614268"/>
+    <sheet name="10A_既設窓互換" sheetId="23" r:id="R78119a376b004a3e"/>
+    <sheet name="10B_現調項目" sheetId="24" r:id="R7d00c7b2c75c4c05"/>
+    <sheet name="99_QA" sheetId="25" r:id="Raac614bf84584871"/>
+    <sheet name="04A_開口構成" sheetId="26" r:id="R874b6fc902ca49ee"/>
+    <sheet name="11_見積入力テスト" sheetId="27" r:id="Re299fc62d7274adb"/>
+    <sheet name="10C_化粧カバー見付" sheetId="28" r:id="R37f3a0b9ef08489f"/>
+    <sheet name="02B_参照商品" sheetId="29" r:id="R2c486cecd873439e"/>
+    <sheet name="02C_新設サッシ手配方式" sheetId="30" r:id="Rd1eb13f484ca4237"/>
+    <sheet name="03C_対応サーモス窓種" sheetId="31" r:id="Rae90d07059364f24"/>
+    <sheet name="03D_サーモス参照制限" sheetId="32" r:id="R096c7adca96149e0"/>
+    <sheet name="05C_寸法変換" sheetId="33" r:id="R525f69380852497b"/>
+    <sheet name="12_共通参照" sheetId="34" r:id="R7af534a981d14c8d"/>
+    <sheet name="02D_対応シリーズ" sheetId="35" r:id="R0774209512b74aa8"/>
+    <sheet name="12A_ATT_TW比較" sheetId="36" r:id="R3603ed6ba51543df"/>
+    <sheet name="13_参照整合性監査" sheetId="37" r:id="R42ed65090b1d4ecf"/>
+    <sheet name="14_UI選択契約" sheetId="38" r:id="rIdReplusUiV9"/>
+  </sheets>
+</workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1442,6 +1443,365 @@
 </a:theme>
 </file>
 
+<file path=xl/worksheets/replus-ui-v9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str" s="244">
+        <v>リプラス住宅用・共通UI選択契約</v>
+      </c>
+      <c r="B1" s="245"/>
+      <c r="C1" s="245"/>
+      <c r="D1" s="245"/>
+      <c r="E1" s="246"/>
+      <c r="F1"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="str" s="241">
+        <v>分類</v>
+      </c>
+      <c r="B2" t="str" s="242">
+        <v>対象</v>
+      </c>
+      <c r="C2" t="str" s="242">
+        <v>依存元</v>
+      </c>
+      <c r="D2" t="str" s="242">
+        <v>処理</v>
+      </c>
+      <c r="E2" t="str" s="243">
+        <v>根拠区分</v>
+      </c>
+      <c r="F2" t="str">
+        <v>revision</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str" s="244">
+        <v>色連動</v>
+      </c>
+      <c r="B3" t="str" s="245">
+        <v>exterior_cover_color</v>
+      </c>
+      <c r="C3" t="str" s="245">
+        <v>new_sash_exterior_color</v>
+      </c>
+      <c r="D3" t="str" s="245">
+        <v>{"targetField": "exterior_cover_color", "parents": ["new_sash_exterior_color"], "cases": [{"when": {"new_sash_exterior_color": "BLACK"}, "value": "T"}, {"when": {"new_sash_exterior_color": "T"}, "value": "T"}, {"when": {"new_sash_exterior_color": "EXT-T"}, "value": "T"}, {"when": {"new_sash_exterior_color": "EXT-LIX-T"}, "value": "T"}, {"when": {"new_sash_exterior_color": "AUTUMN_BROWN"}, "value": "G"}, {"when": {"new_sash_exterior_color": "G"}, "value": "G"}, {"when": {"new_sash_exterior_color": "EXT-G"}, "value": "G"}, {"when": {"new_sash_exterior_color": "EXT-LIX-G"}, "value": "G"}, {"when": {"new_sash_exterior_color": "SHINE_GRAY"}, "value": "K"}, {"when": {"new_sash_exterior_color": "K"}, "value": "K"}, {"when": {"new_sash_exterior_color": "EXT-K"}, "value": "K"}, {"when": {"new_sash_exterior_color": "EXT-LIX-K"}, "value": "K"}, {"when": {"new_sash_exterior_color": "NATURAL_SILVER"}, "value": "D"}, {"when": {"new_sash_exterior_color": "D"}, "value": "D"}, {"when": {"new_sash_exterior_color": "EXT-D"}, "value": "D"}, {"when": {"new_sash_exterior_color": "EXT-LIX-D"}, "value": "D"}, {"when": {"new_sash_exterior_color": "WHITE"}, "value": "W"}, {"when": {"new_sash_exterior_color": "W"}, "value": "W"}, {"when": {"new_sash_exterior_color": "EXT-W"}, "value": "W"}, {"when": {"new_sash_exterior_color": "EXT-LIX-W"}, "value": "W"}], "resolvedMessage": "本体外観色に連動しています。", "pendingMessage": "サッシ本体の色を選択してください。", "unavailableMessage": "本体色に対応するカバー部材の確認が必要です。"}</v>
+      </c>
+      <c r="E3" t="str" s="246">
+        <v>USER_APPLICATION_POLICY</v>
+      </c>
+      <c r="F3" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str" s="244">
+        <v>色連動</v>
+      </c>
+      <c r="B4" t="str" s="245">
+        <v>interior_cover_color</v>
+      </c>
+      <c r="C4" t="str" s="245">
+        <v>new_sash_interior_color</v>
+      </c>
+      <c r="D4" t="str" s="245">
+        <v>{"targetField": "interior_cover_color", "parents": ["new_sash_interior_color"], "cases": [{"when": {"new_sash_interior_color": "BLACK"}, "value": "M"}, {"when": {"new_sash_interior_color": "M"}, "value": "M"}, {"when": {"new_sash_interior_color": "INT-M"}, "value": "M"}, {"when": {"new_sash_interior_color": "INT-LIX-M"}, "value": "M"}, {"when": {"new_sash_interior_color": "AUTUMN_BROWN"}, "value": "G"}, {"when": {"new_sash_interior_color": "G"}, "value": "G"}, {"when": {"new_sash_interior_color": "INT-G"}, "value": "G"}, {"when": {"new_sash_interior_color": "INT-LIX-G"}, "value": "G"}, {"when": {"new_sash_interior_color": "SHINE_GRAY"}, "value": "K"}, {"when": {"new_sash_interior_color": "K"}, "value": "K"}, {"when": {"new_sash_interior_color": "INT-K"}, "value": "K"}, {"when": {"new_sash_interior_color": "INT-LIX-K"}, "value": "K"}, {"when": {"new_sash_interior_color": "NATURAL_SILVER"}, "value": "D"}, {"when": {"new_sash_interior_color": "D"}, "value": "D"}, {"when": {"new_sash_interior_color": "INT-D"}, "value": "D"}, {"when": {"new_sash_interior_color": "INT-LIX-D"}, "value": "D"}, {"when": {"new_sash_interior_color": "WHITE"}, "value": "W"}, {"when": {"new_sash_interior_color": "W"}, "value": "W"}, {"when": {"new_sash_interior_color": "INT-W"}, "value": "W"}, {"when": {"new_sash_interior_color": "INT-LIX-W"}, "value": "W"}, {"when": {"new_sash_interior_color": "CREA_MOCHA"}, "value": "C"}, {"when": {"new_sash_interior_color": "C"}, "value": "C"}, {"when": {"new_sash_interior_color": "INT-C"}, "value": "C"}, {"when": {"new_sash_interior_color": "INT-LIX-C"}, "value": "C"}, {"when": {"new_sash_interior_color": "CREA_RUSK"}, "value": "B"}, {"when": {"new_sash_interior_color": "B"}, "value": "B"}, {"when": {"new_sash_interior_color": "INT-B"}, "value": "B"}, {"when": {"new_sash_interior_color": "INT-LIX-B"}, "value": "B"}, {"when": {"new_sash_interior_color": "CREA_PALE"}, "value": "P"}, {"when": {"new_sash_interior_color": "P"}, "value": "P"}, {"when": {"new_sash_interior_color": "INT-P"}, "value": "P"}, {"when": {"new_sash_interior_color": "INT-LIX-P"}, "value": "P"}, {"when": {"new_sash_interior_color": "PRECIOUS_WHITE"}, "value": "F"}, {"when": {"new_sash_interior_color": "F"}, "value": "F"}, {"when": {"new_sash_interior_color": "INT-F"}, "value": "F"}, {"when": {"new_sash_interior_color": "INT-LIX-F"}, "value": "F"}], "resolvedMessage": "本体内観色に連動しています。", "pendingMessage": "サッシ本体の色を選択してください。", "unavailableMessage": "本体色に対応するカバー部材の確認が必要です。"}</v>
+      </c>
+      <c r="E4" t="str" s="246">
+        <v>USER_APPLICATION_POLICY</v>
+      </c>
+      <c r="F4" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B5" t="str" s="245">
+        <v>referenced_series_id</v>
+      </c>
+      <c r="C5" t="str" s="245"/>
+      <c r="D5" t="str" s="245">
+        <v>{"label": "新設サッシシリーズ", "group": "opening", "internal": false}</v>
+      </c>
+      <c r="E5" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F5" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B6" t="str" s="245">
+        <v>referenced_window_id</v>
+      </c>
+      <c r="C6" t="str" s="245">
+        <v>referenced_series_id</v>
+      </c>
+      <c r="D6" t="str" s="245">
+        <v>{"label": "新設サッシ窓種", "group": "opening", "internal": false}</v>
+      </c>
+      <c r="E6" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F6" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B7" t="str" s="245">
+        <v>exterior_cover_color</v>
+      </c>
+      <c r="C7" t="str" s="245">
+        <v>new_sash_exterior_color</v>
+      </c>
+      <c r="D7" t="str" s="245">
+        <v>{"label": "化粧カバー色（外観色に連動）", "group": "exterior_finish", "internal": false}</v>
+      </c>
+      <c r="E7" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F7" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B8" t="str" s="245">
+        <v>interior_cover_color</v>
+      </c>
+      <c r="C8" t="str" s="245">
+        <v>new_sash_interior_color</v>
+      </c>
+      <c r="D8" t="str" s="245">
+        <v>{"label": "室内カバー色（内観色に連動）", "group": "interior_finish", "internal": false}</v>
+      </c>
+      <c r="E8" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F8" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B9" t="str" s="245">
+        <v>wooden_casing_color</v>
+      </c>
+      <c r="C9" t="str" s="245">
+        <v>options</v>
+      </c>
+      <c r="D9" t="str" s="245">
+        <v>{"label": "木製ケーシング色", "group": "part_detail", "internal": false}</v>
+      </c>
+      <c r="E9" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F9" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B10" t="str" s="245">
+        <v>options</v>
+      </c>
+      <c r="C10" t="str" s="245"/>
+      <c r="D10" t="str" s="245">
+        <v>{"label": "追加部材・オプション", "group": "options", "internal": false}</v>
+      </c>
+      <c r="E10" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F10" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B11" t="str" s="245">
+        <v>survey_w</v>
+      </c>
+      <c r="C11" t="str" s="245"/>
+      <c r="D11" t="str" s="245">
+        <v>{"label": "採寸幅 WS（mm）", "group": "survey", "internal": false}</v>
+      </c>
+      <c r="E11" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F11" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B12" t="str" s="245">
+        <v>survey_h</v>
+      </c>
+      <c r="C12" t="str" s="245"/>
+      <c r="D12" t="str" s="245">
+        <v>{"label": "採寸高さ HS（mm）", "group": "survey", "internal": false}</v>
+      </c>
+      <c r="E12" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F12" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B13" t="str" s="245">
+        <v>existing_frame_depth</v>
+      </c>
+      <c r="C13" t="str" s="245"/>
+      <c r="D13" t="str" s="245">
+        <v>{"label": "既設枠見込み（mm）", "group": "survey", "internal": false}</v>
+      </c>
+      <c r="E13" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F13" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B14" t="str" s="245">
+        <v>lower_frame_rise</v>
+      </c>
+      <c r="C14" t="str" s="245"/>
+      <c r="D14" t="str" s="245">
+        <v>{"label": "既設下枠の立上り（mm）", "group": "survey", "internal": false}</v>
+      </c>
+      <c r="E14" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F14" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B15" t="str" s="245">
+        <v>interior_cover_type</v>
+      </c>
+      <c r="C15" t="str" s="245"/>
+      <c r="D15" t="str" s="245">
+        <v>{"label": "室内側の仕上げ仕様", "group": "interior_finish", "internal": false}</v>
+      </c>
+      <c r="E15" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F15" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B16" t="str" s="245">
+        <v>exterior_cover_type</v>
+      </c>
+      <c r="C16" t="str" s="245">
+        <v>survey_cover_top,survey_cover_bottom,survey_cover_side</v>
+      </c>
+      <c r="D16" t="str" s="245">
+        <v>{"label": "化粧カバーの大きさ・組合せ", "group": "exterior_finish", "internal": false}</v>
+      </c>
+      <c r="E16" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F16" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B17" t="str" s="245">
+        <v>survey_cover_top</v>
+      </c>
+      <c r="C17" t="str" s="245"/>
+      <c r="D17" t="str" s="245">
+        <v>{"label": "既設上枠の見付（mm）", "group": "survey", "internal": false}</v>
+      </c>
+      <c r="E17" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F17" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B18" t="str" s="245">
+        <v>survey_cover_bottom</v>
+      </c>
+      <c r="C18" t="str" s="245"/>
+      <c r="D18" t="str" s="245">
+        <v>{"label": "既設下枠の見付（mm）", "group": "survey", "internal": false}</v>
+      </c>
+      <c r="E18" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F18" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str" s="244">
+        <v>フロー</v>
+      </c>
+      <c r="B19" t="str" s="245">
+        <v>survey_cover_side</v>
+      </c>
+      <c r="C19" t="str" s="245"/>
+      <c r="D19" t="str" s="245">
+        <v>{"label": "既設縦枠の見付（mm）", "group": "survey", "internal": false}</v>
+      </c>
+      <c r="E19" t="str" s="246">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F19" t="str">
+        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
@@ -12033,320 +12393,356 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="76" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="236" t="str">
-        <x:v>01_入力フロー｜アタッチ枠（サーモス用）</x:v>
-      </x:c>
-      <x:c r="B1" s="236"/>
-      <x:c r="C1" s="236"/>
-      <x:c r="D1" s="236"/>
-      <x:c r="E1" s="236"/>
-    </x:row>
-    <x:row r="3" ht="30" customHeight="1">
-      <x:c r="A3" s="241" t="str">
-        <x:v>順序</x:v>
-      </x:c>
-      <x:c r="B3" s="242" t="str">
-        <x:v>表示項目</x:v>
-      </x:c>
-      <x:c r="C3" s="242" t="str">
-        <x:v>データキー</x:v>
-      </x:c>
-      <x:c r="D3" s="242" t="str">
-        <x:v>候補/入力</x:v>
-      </x:c>
-      <x:c r="E3" s="243" t="str">
-        <x:v>制御</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="244" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B4" s="245" t="str">
-        <x:v>取替方式</x:v>
-      </x:c>
-      <x:c r="C4" s="245" t="str">
-        <x:v>installation_system_id</x:v>
-      </x:c>
-      <x:c r="D4" s="245" t="str">
-        <x:v>RPL_ATT_TH</x:v>
-      </x:c>
-      <x:c r="E4" s="246" t="str">
-        <x:v>固定</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="244" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B5" s="245" t="str">
-        <x:v>既設窓条件</x:v>
-      </x:c>
-      <x:c r="C5" s="245" t="str">
-        <x:v>existing_window_compatibility</x:v>
-      </x:c>
-      <x:c r="D5" s="245" t="str">
-        <x:v>既設窓種・材質・構造</x:v>
-      </x:c>
-      <x:c r="E5" s="246" t="str">
-        <x:v>共通ATT適用＋ATT-TH差分</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="244" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B6" s="245" t="str">
-        <x:v>対応シリーズ</x:v>
-      </x:c>
-      <x:c r="C6" s="245" t="str">
-        <x:v>referenced_series_id</x:v>
-      </x:c>
-      <x:c r="D6" s="245" t="str">
-        <x:v>サーモスⅡ-H / サーモスL / サーモスA</x:v>
-      </x:c>
-      <x:c r="E6" s="246" t="str">
-        <x:v>3シリーズとも正本接続済み。ATT-TH公式対応subsetだけ表示</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="244" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B7" s="245" t="str">
-        <x:v>対応窓種</x:v>
-      </x:c>
-      <x:c r="C7" s="245" t="str">
-        <x:v>referenced_window_id</x:v>
-      </x:c>
-      <x:c r="D7" s="245" t="str">
-        <x:v>シリーズ正本から対応窓種だけ</x:v>
-      </x:c>
-      <x:c r="E7" s="246" t="str">
-        <x:v>03Cで絞込</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="244" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B8" s="245" t="str">
-        <x:v>窓種固有仕様</x:v>
-      </x:c>
-      <x:c r="C8" s="245" t="str">
-        <x:v>referenced_spec_selector</x:v>
-      </x:c>
-      <x:c r="D8" s="245" t="str">
-        <x:v>参照先正本</x:v>
-      </x:c>
-      <x:c r="E8" s="246" t="str">
-        <x:v>S2H/L=solid_spec_id、サーモスA=native canonical field/ruleを03Cから適用</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="244" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B9" s="245" t="str">
-        <x:v>施工方法</x:v>
-      </x:c>
-      <x:c r="C9" s="245" t="str">
-        <x:v>installation_method</x:v>
-      </x:c>
-      <x:c r="D9" s="245" t="str">
-        <x:v>STANDARD / INNER_FIT_EXISTING_SINGLE</x:v>
-      </x:c>
-      <x:c r="E9" s="246" t="str">
-        <x:v>既設条件から自動</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="244" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B10" s="245" t="str">
-        <x:v>採寸W/H</x:v>
-      </x:c>
-      <x:c r="C10" s="245" t="str">
-        <x:v>survey_w / survey_h</x:v>
-      </x:c>
-      <x:c r="D10" s="245" t="str">
-        <x:v>3点採寸の最小値</x:v>
-      </x:c>
-      <x:c r="E10" s="246" t="str">
-        <x:v>現調入力</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="244" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B11" s="245" t="str">
-        <x:v>アタッチ枠出来寸</x:v>
-      </x:c>
-      <x:c r="C11" s="245" t="str">
-        <x:v>attachment_finished_w/h</x:v>
-      </x:c>
-      <x:c r="D11" s="245" t="str">
-        <x:v>自動</x:v>
-      </x:c>
-      <x:c r="E11" s="246" t="str">
-        <x:v>WD=WS-10 / HD=HS-10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="244" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B12" s="245" t="str">
-        <x:v>サーモス製作寸法</x:v>
-      </x:c>
-      <x:c r="C12" s="245" t="str">
-        <x:v>referenced_product_w/h</x:v>
-      </x:c>
-      <x:c r="D12" s="245" t="str">
-        <x:v>自動</x:v>
-      </x:c>
-      <x:c r="E12" s="246" t="str">
-        <x:v>W=WS-38 / H=HS-39</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="244" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B13" s="245" t="str">
-        <x:v>参照先サイズ判定</x:v>
-      </x:c>
-      <x:c r="C13" s="245" t="str">
-        <x:v>referenced_size_validation</x:v>
-      </x:c>
-      <x:c r="D13" s="245" t="str">
-        <x:v>サーモス正本へ照会</x:v>
-      </x:c>
-      <x:c r="E13" s="246" t="str">
-        <x:v>本体製作範囲を複製しない</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="244" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B14" s="245" t="str">
-        <x:v>ATT-THローカル判定</x:v>
-      </x:c>
-      <x:c r="C14" s="245" t="str">
-        <x:v>attachment_validation</x:v>
-      </x:c>
-      <x:c r="D14" s="245" t="str">
-        <x:v>W/H包絡・枠見込み・下枠等</x:v>
-      </x:c>
-      <x:c r="E14" s="246" t="str">
-        <x:v>05/10系ルール</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="244" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B15" s="245" t="str">
-        <x:v>サーモス本体仕様</x:v>
-      </x:c>
-      <x:c r="C15" s="245" t="str">
-        <x:v>referenced_product_options</x:v>
-      </x:c>
-      <x:c r="D15" s="245" t="str">
-        <x:v>本体色・網戸・ガラス・OP</x:v>
-      </x:c>
-      <x:c r="E15" s="246" t="str">
-        <x:v>正本から動的取得</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="244" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B16" s="245" t="str">
-        <x:v>化粧カバー</x:v>
-      </x:c>
-      <x:c r="C16" s="245" t="str">
-        <x:v>exterior_cover_type/color</x:v>
-      </x:c>
-      <x:c r="D16" s="245" t="str">
-        <x:v>大/中/小＋5色</x:v>
-      </x:c>
-      <x:c r="E16" s="246" t="str">
-        <x:v>既設見付で絞込</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="244" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B17" s="245" t="str">
-        <x:v>樹脂アングルカバー</x:v>
-      </x:c>
-      <x:c r="C17" s="245" t="str">
-        <x:v>interior_cover_color</x:v>
-      </x:c>
-      <x:c r="D17" s="245" t="str">
-        <x:v>参照内観色から自動/選択</x:v>
-      </x:c>
-      <x:c r="E17" s="246" t="str">
-        <x:v>色互換ルール</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="244" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B18" s="245" t="str">
-        <x:v>リプラス側OP</x:v>
-      </x:c>
-      <x:c r="C18" s="245" t="str">
-        <x:v>attachment_option</x:v>
-      </x:c>
-      <x:c r="D18" s="245" t="str">
-        <x:v>連結ねじ等</x:v>
-      </x:c>
-      <x:c r="E18" s="246" t="str">
-        <x:v>09A依存</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="247" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B19" s="248" t="str">
-        <x:v>最終判定</x:v>
-      </x:c>
-      <x:c r="C19" s="248" t="str">
-        <x:v>final_eligibility</x:v>
-      </x:c>
-      <x:c r="D19" s="248" t="str">
-        <x:v>AUTO / EXTERNAL_CHECK</x:v>
-      </x:c>
-      <x:c r="E19" s="249" t="str">
-        <x:v>参照先判定 AND ATT-TH判定</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:E1"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="58" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="76" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" t="str" s="236">
+        <v>リプラス住宅用・グローバルセレクションフロー</v>
+      </c>
+      <c r="B1" s="236"/>
+      <c r="C1" s="236"/>
+      <c r="D1" s="236"/>
+      <c r="E1" s="236"/>
+      <c r="F1"/>
+    </row>
+    <row r="2">
+      <c r="A2"/>
+      <c r="B2"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" t="str" s="241">
+        <v>順番</v>
+      </c>
+      <c r="B3" t="str" s="242">
+        <v>表示項目</v>
+      </c>
+      <c r="C3" t="str" s="242">
+        <v>データキー</v>
+      </c>
+      <c r="D3" t="str" s="242">
+        <v>候補/入力</v>
+      </c>
+      <c r="E3" t="str" s="243">
+        <v>制御方針</v>
+      </c>
+      <c r="F3"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="244">
+        <v>1</v>
+      </c>
+      <c r="B4" t="str" s="245">
+        <v>商品・リプラス仕様</v>
+      </c>
+      <c r="C4" t="str" s="245">
+        <v>product / specification</v>
+      </c>
+      <c r="D4" t="str" s="245">
+        <v>リプラス住宅用 → 仕様</v>
+      </c>
+      <c r="E4" t="str" s="246">
+        <v>今回承認されたアプリ運用ルール</v>
+      </c>
+      <c r="F4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="244">
+        <v>2</v>
+      </c>
+      <c r="B5" t="str" s="245">
+        <v>設置・施工条件</v>
+      </c>
+      <c r="C5" t="str" s="245">
+        <v>context</v>
+      </c>
+      <c r="D5" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E5" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
+      <c r="F5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="244">
+        <v>3</v>
+      </c>
+      <c r="B6" t="str" s="245">
+        <v>窓種・基本仕様</v>
+      </c>
+      <c r="C6" t="str" s="245">
+        <v>opening</v>
+      </c>
+      <c r="D6" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E6" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
+      <c r="F6"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="244">
+        <v>4</v>
+      </c>
+      <c r="B7" t="str" s="245">
+        <v>本体色</v>
+      </c>
+      <c r="C7" t="str" s="245">
+        <v>finish</v>
+      </c>
+      <c r="D7" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E7" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
+      <c r="F7"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n" s="244">
+        <v>5</v>
+      </c>
+      <c r="B8" t="str" s="245">
+        <v>網戸</v>
+      </c>
+      <c r="C8" t="str" s="245">
+        <v>screen</v>
+      </c>
+      <c r="D8" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E8" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
+      <c r="F8"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="244">
+        <v>6</v>
+      </c>
+      <c r="B9" t="str" s="245">
+        <v>ガラス</v>
+      </c>
+      <c r="C9" t="str" s="245">
+        <v>glazing</v>
+      </c>
+      <c r="D9" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E9" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
+      <c r="F9"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="244">
+        <v>7</v>
+      </c>
+      <c r="B10" t="str" s="245">
+        <v>室内側の仕上げ・アングルカバー</v>
+      </c>
+      <c r="C10" t="str" s="245">
+        <v>interior_finish</v>
+      </c>
+      <c r="D10" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E10" t="str" s="246">
+        <v>本体色に連動</v>
+      </c>
+      <c r="F10"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="244">
+        <v>8</v>
+      </c>
+      <c r="B11" t="str" s="245">
+        <v>室外側の仕上げ・化粧カバー</v>
+      </c>
+      <c r="C11" t="str" s="245">
+        <v>exterior_finish</v>
+      </c>
+      <c r="D11" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E11" t="str" s="246">
+        <v>本体色に連動</v>
+      </c>
+      <c r="F11"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="244">
+        <v>9</v>
+      </c>
+      <c r="B12" t="str" s="245">
+        <v>新設サッシのオプション</v>
+      </c>
+      <c r="C12" t="str" s="245">
+        <v>native_options</v>
+      </c>
+      <c r="D12" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E12" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
+      <c r="F12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="244">
+        <v>10</v>
+      </c>
+      <c r="B13" t="str" s="245">
+        <v>追加部材・オプション</v>
+      </c>
+      <c r="C13" t="str" s="245">
+        <v>options</v>
+      </c>
+      <c r="D13" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E13" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
+      <c r="F13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n" s="244">
+        <v>11</v>
+      </c>
+      <c r="B14" t="str" s="245">
+        <v>選択した部材の仕様</v>
+      </c>
+      <c r="C14" t="str" s="245">
+        <v>part_detail</v>
+      </c>
+      <c r="D14" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E14" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
+      <c r="F14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n" s="244">
+        <v>12</v>
+      </c>
+      <c r="B15" t="str" s="245">
+        <v>現場採寸・取付条件</v>
+      </c>
+      <c r="C15" t="str" s="245">
+        <v>survey</v>
+      </c>
+      <c r="D15" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E15" t="str" s="246">
+        <v>採寸後に再評価</v>
+      </c>
+      <c r="F15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n" s="244">
+        <v>13</v>
+      </c>
+      <c r="B16" t="str" s="245">
+        <v>製品寸法</v>
+      </c>
+      <c r="C16" t="str" s="245">
+        <v>size</v>
+      </c>
+      <c r="D16" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E16" t="str" s="246">
+        <v>採寸後に再評価</v>
+      </c>
+      <c r="F16"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="244"/>
+      <c r="B17" s="245"/>
+      <c r="C17" s="245"/>
+      <c r="D17" s="245"/>
+      <c r="E17" s="246"/>
+      <c r="F17"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="244"/>
+      <c r="B18" s="245"/>
+      <c r="C18" s="245"/>
+      <c r="D18" s="245"/>
+      <c r="E18" s="246"/>
+      <c r="F18"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="247"/>
+      <c r="B19" s="248"/>
+      <c r="C19" s="248"/>
+      <c r="D19" s="248"/>
+      <c r="E19" s="249"/>
+      <c r="F19"/>
+    </row>
+    <row r="20">
+      <c r="A20"/>
+      <c r="B20"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+    </row>
+    <row r="21">
+      <c r="A21"/>
+      <c r="B21"/>
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21"/>
+      <c r="F21"/>
+    </row>
+    <row r="22">
+      <c r="A22"/>
+      <c r="B22"/>
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+      <c r="F22"/>
+    </row>
+    <row r="23">
+      <c r="A23"/>
+      <c r="B23"/>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23"/>
+    </row>
+    <row r="24">
+      <c r="A24"/>
+      <c r="B24"/>
+      <c r="C24"/>
+      <c r="D24"/>
+      <c r="E24"/>
+      <c r="F24"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Remove photographed site inputs from Replus sales selection flow
</commit_message>
<xml_diff>
--- a/changes/replus-runtime-v5/candidates/RPL_ATT_TH.xlsx
+++ b/changes/replus-runtime-v5/candidates/RPL_ATT_TH.xlsx
@@ -1494,7 +1494,7 @@
         <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F3" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="4">
@@ -1514,7 +1514,7 @@
         <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F4" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="5">
@@ -1532,7 +1532,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F5" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="6">
@@ -1552,7 +1552,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F6" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="7">
@@ -1572,7 +1572,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F7" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="8">
@@ -1592,7 +1592,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F8" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="9">
@@ -1612,7 +1612,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F9" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="10">
@@ -1630,7 +1630,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F10" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="11">
@@ -1648,7 +1648,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F11" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="12">
@@ -1666,7 +1666,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F12" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="13">
@@ -1684,7 +1684,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F13" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="14">
@@ -1702,7 +1702,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F14" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="15">
@@ -1720,7 +1720,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F15" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="16">
@@ -1740,7 +1740,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F16" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="17">
@@ -1752,13 +1752,13 @@
       </c>
       <c r="C17" t="str" s="245"/>
       <c r="D17" t="str" s="245">
-        <v>{"label": "既設上枠の見付（mm）", "group": "survey", "internal": false}</v>
+        <v>{"label": "既設上枠の見付（mm）", "group": "survey", "internal": false, "salesInput": false, "required": false, "externalSiteCheck": true}</v>
       </c>
       <c r="E17" t="str" s="246">
-        <v>UI_PRESENTATION</v>
+        <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F17" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="18">
@@ -1770,13 +1770,13 @@
       </c>
       <c r="C18" t="str" s="245"/>
       <c r="D18" t="str" s="245">
-        <v>{"label": "既設下枠の見付（mm）", "group": "survey", "internal": false}</v>
+        <v>{"label": "既設下枠の見付（mm）", "group": "survey", "internal": false, "salesInput": false, "required": false, "externalSiteCheck": true}</v>
       </c>
       <c r="E18" t="str" s="246">
-        <v>UI_PRESENTATION</v>
+        <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F18" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
     <row r="19">
@@ -1788,13 +1788,13 @@
       </c>
       <c r="C19" t="str" s="245"/>
       <c r="D19" t="str" s="245">
-        <v>{"label": "既設縦枠の見付（mm）", "group": "survey", "internal": false}</v>
+        <v>{"label": "既設縦枠の見付（mm）", "group": "survey", "internal": false, "salesInput": false, "required": false, "externalSiteCheck": true}</v>
       </c>
       <c r="E19" t="str" s="246">
-        <v>UI_PRESENTATION</v>
+        <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F19" t="str">
-        <v>REPLUS_GLOBAL_FLOW_V9_20261014</v>
+        <v>REPLUS_SALES_FLOW_V10_20261014</v>
       </c>
     </row>
   </sheetData>
@@ -12462,10 +12462,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="str" s="245">
-        <v>設置・施工条件</v>
+        <v>窓種・基本仕様</v>
       </c>
       <c r="C5" t="str" s="245">
-        <v>context</v>
+        <v>opening</v>
       </c>
       <c r="D5" t="str" s="245">
         <v>選択・確認</v>
@@ -12480,16 +12480,16 @@
         <v>3</v>
       </c>
       <c r="B6" t="str" s="245">
-        <v>窓種・基本仕様</v>
+        <v>室内側の仕上げ・アングルカバー</v>
       </c>
       <c r="C6" t="str" s="245">
-        <v>opening</v>
+        <v>interior_finish</v>
       </c>
       <c r="D6" t="str" s="245">
         <v>選択・確認</v>
       </c>
       <c r="E6" t="str" s="246">
-        <v>対応する項目のみ表示</v>
+        <v>本体色に連動</v>
       </c>
       <c r="F6"/>
     </row>
@@ -12498,16 +12498,16 @@
         <v>4</v>
       </c>
       <c r="B7" t="str" s="245">
-        <v>本体色</v>
+        <v>室外側の仕上げ・化粧カバー</v>
       </c>
       <c r="C7" t="str" s="245">
-        <v>finish</v>
+        <v>exterior_finish</v>
       </c>
       <c r="D7" t="str" s="245">
         <v>選択・確認</v>
       </c>
       <c r="E7" t="str" s="246">
-        <v>対応する項目のみ表示</v>
+        <v>本体色に連動</v>
       </c>
       <c r="F7"/>
     </row>
@@ -12516,10 +12516,10 @@
         <v>5</v>
       </c>
       <c r="B8" t="str" s="245">
-        <v>網戸</v>
+        <v>追加部材・オプション</v>
       </c>
       <c r="C8" t="str" s="245">
-        <v>screen</v>
+        <v>options</v>
       </c>
       <c r="D8" t="str" s="245">
         <v>選択・確認</v>
@@ -12534,10 +12534,10 @@
         <v>6</v>
       </c>
       <c r="B9" t="str" s="245">
-        <v>ガラス</v>
+        <v>選択した部材の仕様</v>
       </c>
       <c r="C9" t="str" s="245">
-        <v>glazing</v>
+        <v>part_detail</v>
       </c>
       <c r="D9" t="str" s="245">
         <v>選択・確認</v>
@@ -12552,125 +12552,65 @@
         <v>7</v>
       </c>
       <c r="B10" t="str" s="245">
-        <v>室内側の仕上げ・アングルカバー</v>
+        <v>現場採寸・取付条件</v>
       </c>
       <c r="C10" t="str" s="245">
-        <v>interior_finish</v>
+        <v>survey</v>
       </c>
       <c r="D10" t="str" s="245">
         <v>選択・確認</v>
       </c>
       <c r="E10" t="str" s="246">
-        <v>本体色に連動</v>
+        <v>採寸後に再評価</v>
       </c>
       <c r="F10"/>
     </row>
     <row r="11">
-      <c r="A11" t="n" s="244">
-        <v>8</v>
-      </c>
-      <c r="B11" t="str" s="245">
-        <v>室外側の仕上げ・化粧カバー</v>
-      </c>
-      <c r="C11" t="str" s="245">
-        <v>exterior_finish</v>
-      </c>
-      <c r="D11" t="str" s="245">
-        <v>選択・確認</v>
-      </c>
-      <c r="E11" t="str" s="246">
-        <v>本体色に連動</v>
-      </c>
+      <c r="A11" s="244"/>
+      <c r="B11" s="245"/>
+      <c r="C11" s="245"/>
+      <c r="D11" s="245"/>
+      <c r="E11" s="246"/>
       <c r="F11"/>
     </row>
     <row r="12">
-      <c r="A12" t="n" s="244">
-        <v>9</v>
-      </c>
-      <c r="B12" t="str" s="245">
-        <v>新設サッシのオプション</v>
-      </c>
-      <c r="C12" t="str" s="245">
-        <v>native_options</v>
-      </c>
-      <c r="D12" t="str" s="245">
-        <v>選択・確認</v>
-      </c>
-      <c r="E12" t="str" s="246">
-        <v>対応する項目のみ表示</v>
-      </c>
+      <c r="A12" s="244"/>
+      <c r="B12" s="245"/>
+      <c r="C12" s="245"/>
+      <c r="D12" s="245"/>
+      <c r="E12" s="246"/>
       <c r="F12"/>
     </row>
     <row r="13">
-      <c r="A13" t="n" s="244">
-        <v>10</v>
-      </c>
-      <c r="B13" t="str" s="245">
-        <v>追加部材・オプション</v>
-      </c>
-      <c r="C13" t="str" s="245">
-        <v>options</v>
-      </c>
-      <c r="D13" t="str" s="245">
-        <v>選択・確認</v>
-      </c>
-      <c r="E13" t="str" s="246">
-        <v>対応する項目のみ表示</v>
-      </c>
+      <c r="A13" s="244"/>
+      <c r="B13" s="245"/>
+      <c r="C13" s="245"/>
+      <c r="D13" s="245"/>
+      <c r="E13" s="246"/>
       <c r="F13"/>
     </row>
     <row r="14">
-      <c r="A14" t="n" s="244">
-        <v>11</v>
-      </c>
-      <c r="B14" t="str" s="245">
-        <v>選択した部材の仕様</v>
-      </c>
-      <c r="C14" t="str" s="245">
-        <v>part_detail</v>
-      </c>
-      <c r="D14" t="str" s="245">
-        <v>選択・確認</v>
-      </c>
-      <c r="E14" t="str" s="246">
-        <v>対応する項目のみ表示</v>
-      </c>
+      <c r="A14" s="244"/>
+      <c r="B14" s="245"/>
+      <c r="C14" s="245"/>
+      <c r="D14" s="245"/>
+      <c r="E14" s="246"/>
       <c r="F14"/>
     </row>
     <row r="15">
-      <c r="A15" t="n" s="244">
-        <v>12</v>
-      </c>
-      <c r="B15" t="str" s="245">
-        <v>現場採寸・取付条件</v>
-      </c>
-      <c r="C15" t="str" s="245">
-        <v>survey</v>
-      </c>
-      <c r="D15" t="str" s="245">
-        <v>選択・確認</v>
-      </c>
-      <c r="E15" t="str" s="246">
-        <v>採寸後に再評価</v>
-      </c>
+      <c r="A15" s="244"/>
+      <c r="B15" s="245"/>
+      <c r="C15" s="245"/>
+      <c r="D15" s="245"/>
+      <c r="E15" s="246"/>
       <c r="F15"/>
     </row>
     <row r="16">
-      <c r="A16" t="n" s="244">
-        <v>13</v>
-      </c>
-      <c r="B16" t="str" s="245">
-        <v>製品寸法</v>
-      </c>
-      <c r="C16" t="str" s="245">
-        <v>size</v>
-      </c>
-      <c r="D16" t="str" s="245">
-        <v>選択・確認</v>
-      </c>
-      <c r="E16" t="str" s="246">
-        <v>採寸後に再評価</v>
-      </c>
+      <c r="A16" s="244"/>
+      <c r="B16" s="245"/>
+      <c r="C16" s="245"/>
+      <c r="D16" s="245"/>
+      <c r="E16" s="246"/>
       <c r="F16"/>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Show measured and finished Replus dimensions and inner-fit selection
</commit_message>
<xml_diff>
--- a/changes/replus-runtime-v5/candidates/RPL_ATT_TH.xlsx
+++ b/changes/replus-runtime-v5/candidates/RPL_ATT_TH.xlsx
@@ -1479,7 +1479,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str" s="244">
-        <v>色連動</v>
+        <v>SELECTION_LINKS</v>
       </c>
       <c r="B3" t="str" s="245">
         <v>exterior_cover_color</v>
@@ -1494,12 +1494,12 @@
         <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F3" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str" s="244">
-        <v>色連動</v>
+        <v>SELECTION_LINKS</v>
       </c>
       <c r="B4" t="str" s="245">
         <v>interior_cover_color</v>
@@ -1514,25 +1514,27 @@
         <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F4" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str" s="244">
-        <v>フロー</v>
+        <v>SELECTION_LINKS</v>
       </c>
       <c r="B5" t="str" s="245">
-        <v>referenced_series_id</v>
-      </c>
-      <c r="C5" t="str" s="245"/>
+        <v>attachment_frame_spec</v>
+      </c>
+      <c r="C5" t="str" s="245">
+        <v>installation_method</v>
+      </c>
       <c r="D5" t="str" s="245">
-        <v>{"label": "新設サッシシリーズ", "group": "opening", "internal": false}</v>
+        <v>{"targetField": "attachment_frame_spec", "parents": ["installation_method"], "cases": [{"when": {"installation_method": "STANDARD"}, "value": "ATT-TH-FRAME-STD"}, {"when": {"installation_method": "INNER_FIT_INSET"}, "value": "ATT-TH-FRAME-INNER-SINGLE"}, {"when": {"installation_method": "INNER_FIT_OUTSET"}, "value": "ATT-TH-FRAME-INNER-SINGLE"}], "resolvedMessage": "施工仕様に連動しています。", "pendingMessage": "内はめ仕様を選択してください。", "unavailableMessage": "アタッチ枠の対応を確認してください。"}</v>
       </c>
       <c r="E5" t="str" s="246">
-        <v>UI_PRESENTATION</v>
+        <v>OFFICIAL_SOURCE_REVIEW</v>
       </c>
       <c r="F5" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="6">
@@ -1540,19 +1542,17 @@
         <v>フロー</v>
       </c>
       <c r="B6" t="str" s="245">
-        <v>referenced_window_id</v>
-      </c>
-      <c r="C6" t="str" s="245">
         <v>referenced_series_id</v>
       </c>
+      <c r="C6" t="str" s="245"/>
       <c r="D6" t="str" s="245">
-        <v>{"label": "新設サッシ窓種", "group": "opening", "internal": false}</v>
+        <v>{"label": "新設サッシシリーズ", "group": "opening", "internal": false}</v>
       </c>
       <c r="E6" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F6" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="7">
@@ -1560,19 +1560,19 @@
         <v>フロー</v>
       </c>
       <c r="B7" t="str" s="245">
-        <v>exterior_cover_color</v>
+        <v>referenced_window_id</v>
       </c>
       <c r="C7" t="str" s="245">
-        <v>new_sash_exterior_color</v>
+        <v>referenced_series_id</v>
       </c>
       <c r="D7" t="str" s="245">
-        <v>{"label": "化粧カバー色（外観色に連動）", "group": "exterior_finish", "internal": false}</v>
+        <v>{"label": "新設サッシ窓種", "group": "opening", "internal": false}</v>
       </c>
       <c r="E7" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F7" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="8">
@@ -1580,19 +1580,19 @@
         <v>フロー</v>
       </c>
       <c r="B8" t="str" s="245">
-        <v>interior_cover_color</v>
+        <v>exterior_cover_color</v>
       </c>
       <c r="C8" t="str" s="245">
-        <v>new_sash_interior_color</v>
+        <v>new_sash_exterior_color</v>
       </c>
       <c r="D8" t="str" s="245">
-        <v>{"label": "室内カバー色（内観色に連動）", "group": "interior_finish", "internal": false}</v>
+        <v>{"label": "化粧カバー色（外観色に連動）", "group": "exterior_finish", "internal": false}</v>
       </c>
       <c r="E8" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F8" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="9">
@@ -1600,19 +1600,19 @@
         <v>フロー</v>
       </c>
       <c r="B9" t="str" s="245">
-        <v>wooden_casing_color</v>
+        <v>interior_cover_color</v>
       </c>
       <c r="C9" t="str" s="245">
-        <v>options</v>
+        <v>new_sash_interior_color</v>
       </c>
       <c r="D9" t="str" s="245">
-        <v>{"label": "木製ケーシング色", "group": "part_detail", "internal": false}</v>
+        <v>{"label": "室内カバー色（内観色に連動）", "group": "interior_finish", "internal": false}</v>
       </c>
       <c r="E9" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F9" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="10">
@@ -1620,17 +1620,19 @@
         <v>フロー</v>
       </c>
       <c r="B10" t="str" s="245">
+        <v>wooden_casing_color</v>
+      </c>
+      <c r="C10" t="str" s="245">
         <v>options</v>
       </c>
-      <c r="C10" t="str" s="245"/>
       <c r="D10" t="str" s="245">
-        <v>{"label": "追加部材・オプション", "group": "options", "internal": false}</v>
+        <v>{"label": "木製ケーシング色", "group": "part_detail", "internal": false}</v>
       </c>
       <c r="E10" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F10" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="11">
@@ -1638,17 +1640,17 @@
         <v>フロー</v>
       </c>
       <c r="B11" t="str" s="245">
-        <v>survey_w</v>
+        <v>options</v>
       </c>
       <c r="C11" t="str" s="245"/>
       <c r="D11" t="str" s="245">
-        <v>{"label": "採寸幅 WS（mm）", "group": "survey", "internal": false}</v>
+        <v>{"label": "追加部材・オプション", "group": "options", "internal": false}</v>
       </c>
       <c r="E11" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F11" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="12">
@@ -1656,17 +1658,17 @@
         <v>フロー</v>
       </c>
       <c r="B12" t="str" s="245">
-        <v>survey_h</v>
+        <v>survey_w</v>
       </c>
       <c r="C12" t="str" s="245"/>
       <c r="D12" t="str" s="245">
-        <v>{"label": "採寸高さ HS（mm）", "group": "survey", "internal": false}</v>
+        <v>{"label": "採寸幅 WS（mm）", "group": "survey", "internal": false}</v>
       </c>
       <c r="E12" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F12" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="13">
@@ -1674,17 +1676,17 @@
         <v>フロー</v>
       </c>
       <c r="B13" t="str" s="245">
-        <v>existing_frame_depth</v>
+        <v>survey_h</v>
       </c>
       <c r="C13" t="str" s="245"/>
       <c r="D13" t="str" s="245">
-        <v>{"label": "既設枠見込み（mm）", "group": "survey", "internal": false}</v>
+        <v>{"label": "採寸高さ HS（mm）", "group": "survey", "internal": false}</v>
       </c>
       <c r="E13" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F13" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="14">
@@ -1692,17 +1694,17 @@
         <v>フロー</v>
       </c>
       <c r="B14" t="str" s="245">
-        <v>lower_frame_rise</v>
+        <v>existing_frame_depth</v>
       </c>
       <c r="C14" t="str" s="245"/>
       <c r="D14" t="str" s="245">
-        <v>{"label": "既設下枠の立上り（mm）", "group": "survey", "internal": false}</v>
+        <v>{"label": "既設枠見込み（mm）", "group": "survey", "internal": false}</v>
       </c>
       <c r="E14" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F14" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="15">
@@ -1710,17 +1712,17 @@
         <v>フロー</v>
       </c>
       <c r="B15" t="str" s="245">
-        <v>interior_cover_type</v>
+        <v>lower_frame_rise</v>
       </c>
       <c r="C15" t="str" s="245"/>
       <c r="D15" t="str" s="245">
-        <v>{"label": "室内側の仕上げ仕様", "group": "interior_finish", "internal": false}</v>
+        <v>{"label": "既設下枠の立上り（mm）", "group": "survey", "internal": false}</v>
       </c>
       <c r="E15" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F15" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="16">
@@ -1728,19 +1730,17 @@
         <v>フロー</v>
       </c>
       <c r="B16" t="str" s="245">
-        <v>exterior_cover_type</v>
-      </c>
-      <c r="C16" t="str" s="245">
-        <v>survey_cover_top,survey_cover_bottom,survey_cover_side</v>
-      </c>
+        <v>interior_cover_type</v>
+      </c>
+      <c r="C16" t="str" s="245"/>
       <c r="D16" t="str" s="245">
-        <v>{"label": "化粧カバーの大きさ・組合せ", "group": "exterior_finish", "internal": false}</v>
+        <v>{"label": "室内側の仕上げ仕様", "group": "interior_finish", "internal": false}</v>
       </c>
       <c r="E16" t="str" s="246">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F16" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="17">
@@ -1748,17 +1748,19 @@
         <v>フロー</v>
       </c>
       <c r="B17" t="str" s="245">
-        <v>survey_cover_top</v>
-      </c>
-      <c r="C17" t="str" s="245"/>
+        <v>exterior_cover_type</v>
+      </c>
+      <c r="C17" t="str" s="245">
+        <v>survey_cover_top,survey_cover_bottom,survey_cover_side</v>
+      </c>
       <c r="D17" t="str" s="245">
-        <v>{"label": "既設上枠の見付（mm）", "group": "survey", "internal": false, "salesInput": false, "required": false, "externalSiteCheck": true}</v>
+        <v>{"label": "化粧カバーの大きさ・組合せ", "group": "exterior_finish", "internal": false}</v>
       </c>
       <c r="E17" t="str" s="246">
-        <v>USER_APPLICATION_POLICY</v>
+        <v>UI_PRESENTATION</v>
       </c>
       <c r="F17" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="18">
@@ -1766,17 +1768,19 @@
         <v>フロー</v>
       </c>
       <c r="B18" t="str" s="245">
-        <v>survey_cover_bottom</v>
-      </c>
-      <c r="C18" t="str" s="245"/>
+        <v>installation_method</v>
+      </c>
+      <c r="C18" t="str" s="245">
+        <v>referenced_window_id</v>
+      </c>
       <c r="D18" t="str" s="245">
-        <v>{"label": "既設下枠の見付（mm）", "group": "survey", "internal": false, "salesInput": false, "required": false, "externalSiteCheck": true}</v>
+        <v>{"label": "内はめ仕様", "group": "inner_fit", "internal": false}</v>
       </c>
       <c r="E18" t="str" s="246">
-        <v>USER_APPLICATION_POLICY</v>
+        <v>UI_PRESENTATION</v>
       </c>
       <c r="F18" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
     <row r="19">
@@ -1784,17 +1788,59 @@
         <v>フロー</v>
       </c>
       <c r="B19" t="str" s="245">
-        <v>survey_cover_side</v>
-      </c>
-      <c r="C19" t="str" s="245"/>
+        <v>attachment_frame_spec</v>
+      </c>
+      <c r="C19" t="str" s="245">
+        <v>installation_method</v>
+      </c>
       <c r="D19" t="str" s="245">
-        <v>{"label": "既設縦枠の見付（mm）", "group": "survey", "internal": false, "salesInput": false, "required": false, "externalSiteCheck": true}</v>
+        <v>{"label": "アタッチ枠仕様", "group": "inner_fit", "internal": false}</v>
       </c>
       <c r="E19" t="str" s="246">
-        <v>USER_APPLICATION_POLICY</v>
+        <v>UI_PRESENTATION</v>
       </c>
       <c r="F19" t="str">
-        <v>REPLUS_SALES_FLOW_V10_20261014</v>
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>フロー</v>
+      </c>
+      <c r="B20" t="str">
+        <v>attachment_finished_w</v>
+      </c>
+      <c r="C20" t="str">
+        <v>survey_w</v>
+      </c>
+      <c r="D20" t="str">
+        <v>{"label": "アタッチ枠仕上がり幅 WD（mm）", "group": "size", "internal": false}</v>
+      </c>
+      <c r="E20" t="str">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F20" t="str">
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>フロー</v>
+      </c>
+      <c r="B21" t="str">
+        <v>attachment_finished_h</v>
+      </c>
+      <c r="C21" t="str">
+        <v>survey_h</v>
+      </c>
+      <c r="D21" t="str">
+        <v>{"label": "アタッチ枠仕上がり高さ HD（mm）", "group": "size", "internal": false}</v>
+      </c>
+      <c r="E21" t="str">
+        <v>UI_PRESENTATION</v>
+      </c>
+      <c r="F21" t="str">
+        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
       </c>
     </row>
   </sheetData>
@@ -1818,7 +1864,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="236" t="str">
+      <c r="A1" t="str" s="236">
         <v>90_Evidence｜ATT-TH v1.1 根拠管理</v>
       </c>
       <c r="B1" s="236"/>
@@ -1831,7 +1877,7 @@
       <c r="I1" s="236"/>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="237" t="str">
+      <c r="A2" t="str" s="237">
         <v>2026-09-01 サーモスA v0.7正本を正式SSOT接続。旧EV-006は履歴として保持しEV-016で更新。</v>
       </c>
       <c r="B2" s="237"/>
@@ -1843,884 +1889,798 @@
       <c r="H2" s="237"/>
       <c r="I2" s="237"/>
     </row>
+    <row r="3">
+      <c r="A3"/>
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3"/>
+    </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="241" t="str">
+      <c r="A4" t="str" s="241">
         <v>evidence_id</v>
       </c>
-      <c r="B4" s="242" t="str">
+      <c r="B4" t="str" s="242">
         <v>情報源種別</v>
       </c>
-      <c r="C4" s="242" t="str">
+      <c r="C4" t="str" s="242">
         <v>資料名</v>
       </c>
-      <c r="D4" s="242" t="str">
+      <c r="D4" t="str" s="242">
         <v>発行年月</v>
       </c>
-      <c r="E4" s="242" t="str">
+      <c r="E4" t="str" s="242">
         <v>ページ/箇所</v>
       </c>
-      <c r="F4" s="242" t="str">
+      <c r="F4" t="str" s="242">
         <v>URL</v>
       </c>
-      <c r="G4" s="242" t="str">
+      <c r="G4" t="str" s="242">
         <v>確認日</v>
       </c>
-      <c r="H4" s="242" t="str">
+      <c r="H4" t="str" s="242">
         <v>確度</v>
       </c>
-      <c r="I4" s="243" t="str">
+      <c r="I4" t="str" s="243">
         <v>根拠内容</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="244" t="str">
+      <c r="A5" t="str" s="244">
         <v>ATT-TH-EV-001</v>
       </c>
-      <c r="B5" s="245" t="str">
+      <c r="B5" t="str" s="245">
         <v>共通仕様</v>
       </c>
-      <c r="C5" s="245" t="str">
+      <c r="C5" t="str" s="245">
         <v>サッシ商品マスター共通仕様書_v0.1</v>
       </c>
-      <c r="D5" s="245" t="str">
+      <c r="D5" t="str" s="245">
         <v>2026-08-30更新</v>
       </c>
-      <c r="E5" s="245" t="str">
+      <c r="E5" t="str" s="245">
         <v>§5,9,23-34</v>
       </c>
-      <c r="F5" s="245" t="str">
+      <c r="F5" t="str" s="245">
         <v>https://docs.google.com/document/d/1MfixkbV1cZ__DtBknEKsix_nnrXQqjc-LZtXUHwJv_A/edit</v>
       </c>
-      <c r="G5" s="245" t="str">
+      <c r="G5" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H5" s="245" t="str">
+      <c r="H5" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I5" s="246" t="str">
+      <c r="I5" t="str" s="246">
         <v>参照型商品マスター、Evidence、UI非表示、耐風圧特殊案件</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="244" t="str">
+      <c r="A6" t="str" s="244">
         <v>ATT-TH-EV-002</v>
       </c>
-      <c r="B6" s="245" t="str">
+      <c r="B6" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C6" s="245" t="str">
+      <c r="C6" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D6" s="245" t="str">
+      <c r="D6" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E6" s="245" t="str">
+      <c r="E6" t="str" s="245">
         <v>p36</v>
       </c>
-      <c r="F6" s="245" t="str">
+      <c r="F6" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G6" s="245" t="str">
+      <c r="G6" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H6" s="245" t="str">
+      <c r="H6" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I6" s="246" t="str">
+      <c r="I6" t="str" s="246">
         <v>ATT-TH概要、対応シリーズS2H/L/A、フィンカット、浴室不可、カバー/アングル色、樹脂/木製既設不可</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="244" t="str">
+      <c r="A7" t="str" s="244">
         <v>ATT-TH-EV-003</v>
       </c>
-      <c r="B7" s="245" t="str">
+      <c r="B7" t="str" s="245">
         <v>商品マスター正本</v>
       </c>
-      <c r="C7" s="245" t="str">
+      <c r="C7" t="str" s="245">
         <v>サーモスⅡH_商品マスター_v0.7_完全完成版.xlsx</v>
       </c>
-      <c r="D7" s="245" t="str">
+      <c r="D7" t="str" s="245">
         <v>現行正本</v>
       </c>
-      <c r="E7" s="245" t="str">
+      <c r="E7" t="str" s="245">
         <v>02_シリーズ/03_窓種/04_窓種固有仕様/06_サイズ</v>
       </c>
-      <c r="F7" s="245" t="str">
+      <c r="F7" t="str" s="245">
         <v>https://docs.google.com/spreadsheets/d/1zHi-XsMqJp0MKH-sDoTcnTqkLMGcuRdo/edit</v>
       </c>
-      <c r="G7" s="245" t="str">
+      <c r="G7" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H7" s="245" t="str">
+      <c r="H7" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I7" s="246" t="str">
+      <c r="I7" t="str" s="246">
         <v>SER-LIX-SAMOS2H、正式window/spec ID、本体サイズ・色・網戸・ガラス・OPのSSOT</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="244" t="str">
+      <c r="A8" t="str" s="244">
         <v>ATT-TH-EV-004</v>
       </c>
-      <c r="B8" s="245" t="str">
+      <c r="B8" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C8" s="245" t="str">
+      <c r="C8" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D8" s="245" t="str">
+      <c r="D8" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E8" s="245" t="str">
+      <c r="E8" t="str" s="245">
         <v>p203</v>
       </c>
-      <c r="F8" s="245" t="str">
+      <c r="F8" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G8" s="245" t="str">
+      <c r="G8" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H8" s="245" t="str">
+      <c r="H8" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I8" s="246" t="str">
+      <c r="I8" t="str" s="246">
         <v>S2H/L/A別対応品種、全シリーズ別途手配＋フィンカット、連結ねじ必須、純正方立/無目不可</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="244" t="str">
+      <c r="A9" t="str" s="244">
         <v>ATT-TH-EV-005</v>
       </c>
-      <c r="B9" s="245" t="str">
+      <c r="B9" t="str" s="245">
         <v>商品マスター正本</v>
       </c>
-      <c r="C9" s="245" t="str">
+      <c r="C9" t="str" s="245">
         <v>サーモスL_商品マスター_v0.7_特注寸法発注アプリ投入完成版_QA確定.xlsx</v>
       </c>
-      <c r="D9" s="245" t="str">
+      <c r="D9" t="str" s="245">
         <v>現行正本</v>
       </c>
-      <c r="E9" s="245" t="str">
+      <c r="E9" t="str" s="245">
         <v>02_シリーズ/03_窓種/04_窓種固有仕様/06_サイズ</v>
       </c>
-      <c r="F9" s="245" t="str">
+      <c r="F9" t="str" s="245">
         <v>https://docs.google.com/spreadsheets/d/17lVzBZ1hp4RVcGv0yNdnrKt25SFO2FhL/edit</v>
       </c>
-      <c r="G9" s="245" t="str">
+      <c r="G9" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H9" s="245" t="str">
+      <c r="H9" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I9" s="246" t="str">
+      <c r="I9" t="str" s="246">
         <v>SER-LIX-SAMOSL、正式window/spec ID、本体仕様SSOT</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="244" t="str">
+      <c r="A10" t="str" s="244">
         <v>ATT-TH-EV-006</v>
       </c>
-      <c r="B10" s="245" t="str">
+      <c r="B10" t="str" s="245">
         <v>Drive正本確認</v>
       </c>
-      <c r="C10" s="245" t="str">
+      <c r="C10" t="str" s="245">
         <v>04_商品マスター/01_LIXIL</v>
       </c>
-      <c r="D10" s="245" t="str">
+      <c r="D10" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="E10" s="245" t="str">
+      <c r="E10" t="str" s="245">
         <v>フォルダ一覧</v>
       </c>
-      <c r="F10" s="245" t="str">
+      <c r="F10" t="str" s="245">
         <v>https://drive.google.com/drive/folders/1TPaSG9ufcfOZISRXlvOW38JuUu01xqjH</v>
       </c>
-      <c r="G10" s="245" t="str">
+      <c r="G10" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H10" s="245" t="str">
+      <c r="H10" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I10" s="246" t="str">
+      <c r="I10" t="str" s="246">
         <v>2026-08-31時点の履歴：当時サーモスA正本未存在。2026-09-01のATT-TH-EV-016でSUPERSEDED。</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="244" t="str">
+      <c r="A11" t="str" s="244">
         <v>ATT-TH-EV-007</v>
       </c>
-      <c r="B11" s="245" t="str">
+      <c r="B11" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C11" s="245" t="str">
+      <c r="C11" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D11" s="245" t="str">
+      <c r="D11" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E11" s="245" t="str">
+      <c r="E11" t="str" s="245">
         <v>p88価格表/p189基本寸法</v>
       </c>
-      <c r="F11" s="245" t="str">
+      <c r="F11" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G11" s="245" t="str">
+      <c r="G11" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H11" s="245" t="str">
+      <c r="H11" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I11" s="246" t="str">
+      <c r="I11" t="str" s="246">
         <v>WD=WS-10、HD=HS-10、Thermos_W=WS-38、Thermos_H=HS-39</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="244" t="str">
+      <c r="A12" t="str" s="244">
         <v>ATT-TH-EV-008</v>
       </c>
-      <c r="B12" s="245" t="str">
+      <c r="B12" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C12" s="245" t="str">
+      <c r="C12" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D12" s="245" t="str">
+      <c r="D12" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E12" s="245" t="str">
+      <c r="E12" t="str" s="245">
         <v>p196-210 現場調査</v>
       </c>
-      <c r="F12" s="245" t="str">
+      <c r="F12" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G12" s="245" t="str">
+      <c r="G12" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H12" s="245" t="str">
+      <c r="H12" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I12" s="246" t="str">
+      <c r="I12" t="str" s="246">
         <v>ATT-TW/TH共通の建物/既設窓/3点採寸/二重サッシ等</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="244" t="str">
+      <c r="A13" t="str" s="244">
         <v>ATT-TH-EV-009</v>
       </c>
-      <c r="B13" s="245" t="str">
+      <c r="B13" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C13" s="245" t="str">
+      <c r="C13" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D13" s="245" t="str">
+      <c r="D13" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E13" s="245" t="str">
+      <c r="E13" t="str" s="245">
         <v>p201</v>
       </c>
-      <c r="F13" s="245" t="str">
+      <c r="F13" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G13" s="245" t="str">
+      <c r="G13" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H13" s="245" t="str">
+      <c r="H13" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I13" s="246" t="str">
+      <c r="I13" t="str" s="246">
         <v>ATT-TH既設枠見込み寸法90mm以下</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="244" t="str">
+      <c r="A14" t="str" s="244">
         <v>ATT-TH-EV-010</v>
       </c>
-      <c r="B14" s="245" t="str">
+      <c r="B14" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C14" s="245" t="str">
+      <c r="C14" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D14" s="245" t="str">
+      <c r="D14" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E14" s="245" t="str">
+      <c r="E14" t="str" s="245">
         <v>p209</v>
       </c>
-      <c r="F14" s="245" t="str">
+      <c r="F14" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G14" s="245" t="str">
+      <c r="G14" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H14" s="245" t="str">
+      <c r="H14" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I14" s="246" t="str">
+      <c r="I14" t="str" s="246">
         <v>下枠補強金具34～53mm、min/max外スペーサー対応、装飾窓W&lt;=800は補強確認不要</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="244" t="str">
+      <c r="A15" t="str" s="244">
         <v>ATT-TH-EV-011</v>
       </c>
-      <c r="B15" s="245" t="str">
+      <c r="B15" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C15" s="245" t="str">
+      <c r="C15" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D15" s="245" t="str">
+      <c r="D15" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E15" s="245" t="str">
+      <c r="E15" t="str" s="245">
         <v>p211</v>
       </c>
-      <c r="F15" s="245" t="str">
+      <c r="F15" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G15" s="245" t="str">
+      <c r="G15" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H15" s="245" t="str">
+      <c r="H15" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I15" s="246" t="str">
+      <c r="I15" t="str" s="246">
         <v>ATT-TH化粧カバー見付 大71.5/96/34、中36.5/61/34、小16.5/41/9</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="244" t="str">
+      <c r="A16" t="str" s="244">
         <v>ATT-TH-EV-012</v>
       </c>
-      <c r="B16" s="245" t="str">
+      <c r="B16" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C16" s="245" t="str">
+      <c r="C16" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D16" s="245" t="str">
+      <c r="D16" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E16" s="245" t="str">
+      <c r="E16" t="str" s="245">
         <v>p88-89,p136-138</v>
       </c>
-      <c r="F16" s="245" t="str">
+      <c r="F16" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G16" s="245" t="str">
+      <c r="G16" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H16" s="245" t="str">
+      <c r="H16" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I16" s="246" t="str">
+      <c r="I16" t="str" s="246">
         <v>ATT-TH部材価格/製作包絡、専用連窓方立・段窓無目、総W/総H式、純正方立/無目使用不可</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="244" t="str">
+      <c r="A17" t="str" s="244">
         <v>ATT-TH-EV-013</v>
       </c>
-      <c r="B17" s="245" t="str">
+      <c r="B17" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C17" s="245" t="str">
+      <c r="C17" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D17" s="245" t="str">
+      <c r="D17" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E17" s="245" t="str">
+      <c r="E17" t="str" s="245">
         <v>p72-73,p90-92</v>
       </c>
-      <c r="F17" s="245" t="str">
+      <c r="F17" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G17" s="245" t="str">
+      <c r="G17" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H17" s="245" t="str">
+      <c r="H17" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I17" s="246" t="str">
+      <c r="I17" t="str" s="246">
         <v>連結ねじ、気密テープ、充てん材、ケーシング、施工スペーサー等の有償品対応</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="244" t="str">
+      <c r="A18" t="str" s="244">
         <v>ATT-TH-EV-014</v>
       </c>
-      <c r="B18" s="245" t="str">
+      <c r="B18" t="str" s="245">
         <v>商品カタログ</v>
       </c>
-      <c r="C18" s="245" t="str">
+      <c r="C18" t="str" s="245">
         <v>LIXIL リプラス 商品カタログ</v>
       </c>
-      <c r="D18" s="245" t="str">
+      <c r="D18" t="str" s="245">
         <v>2025-08</v>
       </c>
-      <c r="E18" s="245" t="str">
+      <c r="E18" t="str" s="245">
         <v>p263-264</v>
       </c>
-      <c r="F18" s="245" t="str">
+      <c r="F18" t="str" s="245">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G18" s="245" t="str">
+      <c r="G18" t="str" s="245">
         <v>2026-08-31</v>
       </c>
-      <c r="H18" s="245" t="str">
+      <c r="H18" t="str" s="245">
         <v>HIGH</v>
       </c>
-      <c r="I18" s="246" t="str">
+      <c r="I18" t="str" s="246">
         <v>ATT-TH部材詳細：標準/既設単体内嵌め用、化粧カバー、アングルカバー、見切材</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="247" t="str">
+      <c r="A19" t="str" s="247">
         <v>ATT-TH-EV-015</v>
       </c>
-      <c r="B19" s="248" t="str">
+      <c r="B19" t="str" s="248">
         <v>商品カタログ/業務用資料</v>
       </c>
-      <c r="C19" s="248" t="str">
+      <c r="C19" t="str" s="248">
         <v>リプラス公式資料</v>
       </c>
-      <c r="D19" s="248" t="str">
+      <c r="D19" t="str" s="248">
         <v>2025-08/2026-04</v>
       </c>
-      <c r="E19" s="248" t="str">
+      <c r="E19" t="str" s="248">
         <v>p138,p142/特殊性能・施工注意</v>
       </c>
-      <c r="F19" s="248" t="str">
+      <c r="F19" t="str" s="248">
         <v>https://drive.google.com/file/d/1D1HPMXhOMYd_Lu10XNzzJR2TH3aDHVUr/view</v>
       </c>
-      <c r="G19" s="248" t="str">
+      <c r="G19" t="str" s="248">
         <v>2026-08-31</v>
       </c>
-      <c r="H19" s="248" t="str">
+      <c r="H19" t="str" s="248">
         <v>HIGH</v>
       </c>
-      <c r="I19" s="249" t="str">
+      <c r="I19" t="str" s="249">
         <v>内嵌め図形、耐風圧、連段特殊境界、施工スペース・屋外建込み条件は外部/現場確認</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="38" t="str">
+      <c r="A20" t="str" s="38">
         <v>ATT-TH-EV-016</v>
       </c>
-      <c r="B20" s="39" t="str">
+      <c r="B20" t="str" s="39">
         <v>商品マスター正本</v>
       </c>
-      <c r="C20" s="39" t="str">
+      <c r="C20" t="str" s="39">
         <v>サーモスA_商品マスター_v0.7.xlsx</v>
       </c>
-      <c r="D20" s="39" t="str">
+      <c r="D20" t="str" s="39">
         <v>v0.7</v>
       </c>
-      <c r="E20" s="39" t="str">
+      <c r="E20" t="str" s="39">
         <v>00_RELEASE_MANIFEST / 01_SERIES_MASTER / 02_WINDOW_TYPE_MASTER / 14_SIZE_AVAILABILITY / 15_DEPENDENCY_RULE / 20_RULE_BUNDLE / 21_GOLDEN_TEST / 90_QA_SUMMARY</v>
       </c>
-      <c r="F20" s="39" t="str">
+      <c r="F20" t="str" s="39">
         <v>https://docs.google.com/spreadsheets/d/1cDEFzi0g1DzM5YoeGvZtHuXionD7tmFD/edit</v>
       </c>
-      <c r="G20" s="39" t="str">
+      <c r="G20" t="str" s="39">
         <v>2026-09-01</v>
       </c>
-      <c r="H20" s="39" t="str">
+      <c r="H20" t="str" s="39">
         <v>HIGH</v>
       </c>
-      <c r="I20" s="40" t="str">
+      <c r="I20" t="str" s="40">
         <v>Drive file ID=1cDEFzi0g1DzM5YoeGvZtHuXionD7tmFD; series_id=SER-LIX-SAMOSA; APP_READY/QA_PASS; Golden Test 40/40 PASS; active window types and runtime resolve_size contract confirmed.</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="str">
+      <c r="A21" t="str" s="28">
         <v>ATT-TH-EV-017</v>
       </c>
-      <c r="B21" s="28" t="str">
+      <c r="B21" t="str" s="28">
         <v>公式対応突合</v>
       </c>
-      <c r="C21" s="28" t="str">
+      <c r="C21" t="str" s="28">
         <v>LIXIL リプラス 商品カタログ × サーモスA v0.7正本</v>
       </c>
-      <c r="D21" s="28" t="str">
+      <c r="D21" t="str" s="28">
         <v>2025-08 / v0.7</v>
       </c>
-      <c r="E21" s="28" t="str">
+      <c r="E21" t="str" s="28">
         <v>リプラス p203 × SAMOSA 02_WINDOW_TYPE_MASTER/15_DEPENDENCY_RULE</v>
       </c>
-      <c r="F21" s="28" t="str">
+      <c r="F21" t="str" s="28">
         <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
       </c>
-      <c r="G21" s="28" t="str">
+      <c r="G21" t="str" s="28">
         <v>2026-09-01</v>
       </c>
-      <c r="H21" s="28" t="str">
+      <c r="H21" t="str" s="28">
         <v>HIGH</v>
       </c>
-      <c r="I21" s="28" t="str">
+      <c r="I21" t="str" s="28">
         <v>ATT-TH×サーモスA対応subsetを正式IDへ突合：WT-SA-TATE-SUBERI(T+cam_latch), WT-SA-YOKO-SUBERI(cam_latch), WT-SA-KOSHO-YOKO, WT-SA-FIX-IN, WT-SA-UCHIDAOSHI, WT-SA-SOTODAOSHI。solid_spec_idはSAMOSA正本に存在せずnative fields/rulesで表現。</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="str">
+      <c r="A22" t="str" s="28">
         <v>ATT-TH-EV-018</v>
       </c>
-      <c r="B22" s="28" t="str">
+      <c r="B22" t="str" s="28">
         <v>版管理</v>
       </c>
-      <c r="C22" s="28" t="str">
+      <c r="C22" t="str" s="28">
         <v>サッシ商品マスター_保管・版管理仕様書_v1.0</v>
       </c>
-      <c r="D22" s="28" t="str">
+      <c r="D22" t="str" s="28">
         <v>v1.0</v>
       </c>
-      <c r="E22" s="28" t="str">
+      <c r="E22" t="str" s="28">
         <v>§6-10 正本・旧版・version運用</v>
       </c>
-      <c r="F22" s="28" t="str">
+      <c r="F22" t="str" s="28">
         <v>https://docs.google.com/document/d/181yiJ0Ub3t2YdkZ2nx5kagahnB8H8r4RKQRRpQttqNw/edit</v>
       </c>
-      <c r="G22" s="28" t="str">
+      <c r="G22" t="str" s="28">
         <v>2026-09-01</v>
       </c>
-      <c r="H22" s="28" t="str">
+      <c r="H22" t="str" s="28">
         <v>HIGH</v>
       </c>
-      <c r="I22" s="28" t="str">
+      <c r="I22" t="str" s="28">
         <v>データ追加・参照接続・QA反映はマイナーversion更新。ATT-TH v1.0を履歴保持し、v1.1を新採用版として作成。</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
-        <is>
-          <t>DELTA-SPACER-EV-V4</t>
-        </is>
-      </c>
-      <c r="B23" s="28" t="inlineStr">
-        <is>
-          <t>公式業務用資料集</t>
-        </is>
-      </c>
-      <c r="C23" s="28" t="inlineStr">
-        <is>
-          <t>IS9800</t>
-        </is>
-      </c>
-      <c r="D23" s="28" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="E23" s="28" t="inlineStr">
-        <is>
-          <t>PDF 52,104,116,120</t>
-        </is>
-      </c>
-      <c r="F23" s="28" t="inlineStr">
-        <is>
-          <t>https://webcatalog.lixil.co.jp/cgi-bin/openCatalog.cgi?c=IS9800&amp;d=newinter</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="H23" s="28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="I23" s="28" t="inlineStr">
-        <is>
-          <t>ADD_15x20_SPACER / NEW_CANDIDATE、Current未採用</t>
-        </is>
+      <c r="A23" t="str" s="28">
+        <v>DELTA-SPACER-EV-V4</v>
+      </c>
+      <c r="B23" t="str" s="28">
+        <v>公式業務用資料集</v>
+      </c>
+      <c r="C23" t="str" s="28">
+        <v>IS9800</v>
+      </c>
+      <c r="D23" t="str" s="28">
+        <v>2026-10</v>
+      </c>
+      <c r="E23" t="str" s="28">
+        <v>PDF 52,104,116,120</v>
+      </c>
+      <c r="F23" t="str" s="28">
+        <v>https://webcatalog.lixil.co.jp/cgi-bin/openCatalog.cgi?c=IS9800&amp;d=newinter</v>
+      </c>
+      <c r="G23" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="H23" t="str" s="28">
+        <v>HIGH</v>
+      </c>
+      <c r="I23" t="str" s="28">
+        <v>ADD_15x20_SPACER / NEW_CANDIDATE、Current未採用</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="inlineStr">
-        <is>
-          <t>DELTA-CASING-EV-V4</t>
-        </is>
-      </c>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>公式業務用資料集</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="inlineStr">
-        <is>
-          <t>IS9800</t>
-        </is>
-      </c>
-      <c r="D24" s="28" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="E24" s="28" t="inlineStr">
-        <is>
-          <t>PDF 51,115,119</t>
-        </is>
-      </c>
-      <c r="F24" s="28" t="inlineStr">
-        <is>
-          <t>https://webcatalog.lixil.co.jp/cgi-bin/openCatalog.cgi?c=IS9800&amp;d=newinter</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="H24" s="28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="I24" s="28" t="inlineStr">
-        <is>
-          <t>UPDATE_WOODEN_CASING_COLOR_SCOPE / NEW_CANDIDATE、Current未採用</t>
-        </is>
+      <c r="A24" t="str" s="28">
+        <v>DELTA-CASING-EV-V4</v>
+      </c>
+      <c r="B24" t="str" s="28">
+        <v>公式業務用資料集</v>
+      </c>
+      <c r="C24" t="str" s="28">
+        <v>IS9800</v>
+      </c>
+      <c r="D24" t="str" s="28">
+        <v>2026-10</v>
+      </c>
+      <c r="E24" t="str" s="28">
+        <v>PDF 51,115,119</v>
+      </c>
+      <c r="F24" t="str" s="28">
+        <v>https://webcatalog.lixil.co.jp/cgi-bin/openCatalog.cgi?c=IS9800&amp;d=newinter</v>
+      </c>
+      <c r="G24" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="H24" t="str" s="28">
+        <v>HIGH</v>
+      </c>
+      <c r="I24" t="str" s="28">
+        <v>UPDATE_WOODEN_CASING_COLOR_SCOPE / NEW_CANDIDATE、Current未採用</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="inlineStr">
-        <is>
-          <t>DELTA-FILLER-EV-V4</t>
-        </is>
-      </c>
-      <c r="B25" s="28" t="inlineStr">
-        <is>
-          <t>公式業務用資料集</t>
-        </is>
-      </c>
-      <c r="C25" s="28" t="inlineStr">
-        <is>
-          <t>IS9800</t>
-        </is>
-      </c>
-      <c r="D25" s="28" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="E25" s="28" t="inlineStr">
-        <is>
-          <t>PDF 51,115,119</t>
-        </is>
-      </c>
-      <c r="F25" s="28" t="inlineStr">
-        <is>
-          <t>https://webcatalog.lixil.co.jp/cgi-bin/openCatalog.cgi?c=IS9800&amp;d=newinter</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="H25" s="28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="I25" s="28" t="inlineStr">
-        <is>
-          <t>UPDATE_FILLER_NAME_AND_VARIANTS / NEW_CANDIDATE、Current未採用</t>
-        </is>
+      <c r="A25" t="str" s="28">
+        <v>DELTA-FILLER-EV-V4</v>
+      </c>
+      <c r="B25" t="str" s="28">
+        <v>公式業務用資料集</v>
+      </c>
+      <c r="C25" t="str" s="28">
+        <v>IS9800</v>
+      </c>
+      <c r="D25" t="str" s="28">
+        <v>2026-10</v>
+      </c>
+      <c r="E25" t="str" s="28">
+        <v>PDF 51,115,119</v>
+      </c>
+      <c r="F25" t="str" s="28">
+        <v>https://webcatalog.lixil.co.jp/cgi-bin/openCatalog.cgi?c=IS9800&amp;d=newinter</v>
+      </c>
+      <c r="G25" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="H25" t="str" s="28">
+        <v>HIGH</v>
+      </c>
+      <c r="I25" t="str" s="28">
+        <v>UPDATE_FILLER_NAME_AND_VARIANTS / NEW_CANDIDATE、Current未採用</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="inlineStr">
-        <is>
-          <t>DELTA-LEADTIME-EV-V4</t>
-        </is>
-      </c>
-      <c r="B26" s="28" t="inlineStr">
-        <is>
-          <t>公式業務用資料集</t>
-        </is>
-      </c>
-      <c r="C26" s="28" t="inlineStr">
-        <is>
-          <t>IS9800</t>
-        </is>
-      </c>
-      <c r="D26" s="28" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="E26" s="28" t="inlineStr">
-        <is>
-          <t>PDF 235</t>
-        </is>
-      </c>
-      <c r="F26" s="28" t="inlineStr">
-        <is>
-          <t>https://webcatalog.lixil.co.jp/cgi-bin/openCatalog.cgi?c=IS9800&amp;d=newinter</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="H26" s="28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="I26" s="28" t="inlineStr">
-        <is>
-          <t>SOURCE_NOTE_ONLY / NEW_CANDIDATE、Current未採用</t>
-        </is>
+      <c r="A26" t="str" s="28">
+        <v>DELTA-LEADTIME-EV-V4</v>
+      </c>
+      <c r="B26" t="str" s="28">
+        <v>公式業務用資料集</v>
+      </c>
+      <c r="C26" t="str" s="28">
+        <v>IS9800</v>
+      </c>
+      <c r="D26" t="str" s="28">
+        <v>2026-10</v>
+      </c>
+      <c r="E26" t="str" s="28">
+        <v>PDF 235</v>
+      </c>
+      <c r="F26" t="str" s="28">
+        <v>https://webcatalog.lixil.co.jp/cgi-bin/openCatalog.cgi?c=IS9800&amp;d=newinter</v>
+      </c>
+      <c r="G26" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="H26" t="str" s="28">
+        <v>HIGH</v>
+      </c>
+      <c r="I26" t="str" s="28">
+        <v>SOURCE_NOTE_ONLY / NEW_CANDIDATE、Current未採用</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
-        <is>
-          <t>REF-S2-CURRENT-20261009-V4</t>
-        </is>
-      </c>
-      <c r="B27" s="28" t="inlineStr">
-        <is>
-          <t>Current正本参照</t>
-        </is>
-      </c>
-      <c r="C27" s="28" t="inlineStr">
-        <is>
-          <t>v0.9-R4 Current Authoring</t>
-        </is>
-      </c>
-      <c r="D27" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E27" s="28" t="inlineStr">
-        <is>
-          <t>固定参照ID/SHA</t>
-        </is>
-      </c>
-      <c r="F27" s="28" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1_p-xJ9Mv7FecoR8Me0E43f3LEEkpVQSP/view</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="H27" s="28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="I27" s="28" t="inlineStr">
-        <is>
-          <t>eeb285689a1e8a78469d5d13d1e015083d7f2e71ab274427dcfd413e33adc8e4</t>
-        </is>
+      <c r="A27" t="str" s="28">
+        <v>REF-S2-CURRENT-20261009-V4</v>
+      </c>
+      <c r="B27" t="str" s="28">
+        <v>Current正本参照</v>
+      </c>
+      <c r="C27" t="str" s="28">
+        <v>v0.9-R4 Current Authoring</v>
+      </c>
+      <c r="D27" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="E27" t="str" s="28">
+        <v>固定参照ID/SHA</v>
+      </c>
+      <c r="F27" t="str" s="28">
+        <v>https://drive.google.com/file/d/1_p-xJ9Mv7FecoR8Me0E43f3LEEkpVQSP/view</v>
+      </c>
+      <c r="G27" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="H27" t="str" s="28">
+        <v>HIGH</v>
+      </c>
+      <c r="I27" t="str" s="28">
+        <v>eeb285689a1e8a78469d5d13d1e015083d7f2e71ab274427dcfd413e33adc8e4</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
-        <is>
-          <t>REF-SL-CURRENT-20261009-V4</t>
-        </is>
-      </c>
-      <c r="B28" s="28" t="inlineStr">
-        <is>
-          <t>Current正本参照</t>
-        </is>
-      </c>
-      <c r="C28" s="28" t="inlineStr">
-        <is>
-          <t>v0.7-R3 Current Authoring</t>
-        </is>
-      </c>
-      <c r="D28" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E28" s="28" t="inlineStr">
-        <is>
-          <t>固定参照ID/SHA</t>
-        </is>
-      </c>
-      <c r="F28" s="28" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/19sjSAPwyd30fF5akazldGs0wkhOGZF9v/view</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="H28" s="28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="I28" s="28" t="inlineStr">
-        <is>
-          <t>42a1a159c199ac0290f4862b20381abf2450b686ae8a8a2abdaa2d428a8c73f8</t>
-        </is>
+      <c r="A28" t="str" s="28">
+        <v>REF-SL-CURRENT-20261009-V4</v>
+      </c>
+      <c r="B28" t="str" s="28">
+        <v>Current正本参照</v>
+      </c>
+      <c r="C28" t="str" s="28">
+        <v>v0.7-R3 Current Authoring</v>
+      </c>
+      <c r="D28" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="E28" t="str" s="28">
+        <v>固定参照ID/SHA</v>
+      </c>
+      <c r="F28" t="str" s="28">
+        <v>https://drive.google.com/file/d/19sjSAPwyd30fF5akazldGs0wkhOGZF9v/view</v>
+      </c>
+      <c r="G28" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="H28" t="str" s="28">
+        <v>HIGH</v>
+      </c>
+      <c r="I28" t="str" s="28">
+        <v>42a1a159c199ac0290f4862b20381abf2450b686ae8a8a2abdaa2d428a8c73f8</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="inlineStr">
-        <is>
-          <t>REF-A-CURRENT-20261009-V4</t>
-        </is>
-      </c>
-      <c r="B29" s="28" t="inlineStr">
-        <is>
-          <t>Current正本参照</t>
-        </is>
-      </c>
-      <c r="C29" s="28" t="inlineStr">
-        <is>
-          <t>v0.7 Current Authoring</t>
-        </is>
-      </c>
-      <c r="D29" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E29" s="28" t="inlineStr">
-        <is>
-          <t>固定参照ID/SHA</t>
-        </is>
-      </c>
-      <c r="F29" s="28" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1cDEFzi0g1DzM5YoeGvZtHuXionD7tmFD/view</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="H29" s="28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="I29" s="28" t="inlineStr">
-        <is>
-          <t>1aae676ab404e9110ec6bb5aab522c6c0dc2fdc856a0d7c734fd2561fc5dfe47</t>
-        </is>
+      <c r="A29" t="str" s="28">
+        <v>REF-A-CURRENT-20261009-V4</v>
+      </c>
+      <c r="B29" t="str" s="28">
+        <v>Current正本参照</v>
+      </c>
+      <c r="C29" t="str" s="28">
+        <v>v0.7 Current Authoring</v>
+      </c>
+      <c r="D29" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="E29" t="str" s="28">
+        <v>固定参照ID/SHA</v>
+      </c>
+      <c r="F29" t="str" s="28">
+        <v>https://drive.google.com/file/d/1cDEFzi0g1DzM5YoeGvZtHuXionD7tmFD/view</v>
+      </c>
+      <c r="G29" t="str" s="28">
+        <v>2026-10-14</v>
+      </c>
+      <c r="H29" t="str" s="28">
+        <v>HIGH</v>
+      </c>
+      <c r="I29" t="str" s="28">
+        <v>1aae676ab404e9110ec6bb5aab522c6c0dc2fdc856a0d7c734fd2561fc5dfe47</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>EV-DIMENSIONS-INNER-FIT-V11</v>
+      </c>
+      <c r="B30" t="str">
+        <v>公式商品カタログ</v>
+      </c>
+      <c r="C30" t="str">
+        <v>リプラス SN1200</v>
+      </c>
+      <c r="D30" t="str">
+        <v>2025-08</v>
+      </c>
+      <c r="E30" t="str">
+        <v>PDF252/254・231/233/247/249/251</v>
+      </c>
+      <c r="F30" t="str">
+        <v>https://drive.google.com/file/d/1wH1nhmsftl6y8Mp7y6twtoXSi6rxqxzT/view</v>
+      </c>
+      <c r="G30" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="H30" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="I30" t="str">
+        <v>採寸/出来寸の相互換算と標準/内はめの施工仕様を共通Runtimeへ接続</v>
       </c>
     </row>
   </sheetData>
@@ -12453,7 +12413,7 @@
         <v>リプラス住宅用 → 仕様</v>
       </c>
       <c r="E4" t="str" s="246">
-        <v>今回承認されたアプリ運用ルール</v>
+        <v>アプリ運用ルール</v>
       </c>
       <c r="F4"/>
     </row>
@@ -12480,16 +12440,16 @@
         <v>3</v>
       </c>
       <c r="B6" t="str" s="245">
-        <v>室内側の仕上げ・アングルカバー</v>
+        <v>内はめ仕様</v>
       </c>
       <c r="C6" t="str" s="245">
-        <v>interior_finish</v>
+        <v>inner_fit</v>
       </c>
       <c r="D6" t="str" s="245">
         <v>選択・確認</v>
       </c>
       <c r="E6" t="str" s="246">
-        <v>本体色に連動</v>
+        <v>ガラスの後で選択</v>
       </c>
       <c r="F6"/>
     </row>
@@ -12498,16 +12458,16 @@
         <v>4</v>
       </c>
       <c r="B7" t="str" s="245">
-        <v>室外側の仕上げ・化粧カバー</v>
+        <v>室内側の仕上げ・アングルカバー</v>
       </c>
       <c r="C7" t="str" s="245">
-        <v>exterior_finish</v>
+        <v>interior_finish</v>
       </c>
       <c r="D7" t="str" s="245">
         <v>選択・確認</v>
       </c>
       <c r="E7" t="str" s="246">
-        <v>本体色に連動</v>
+        <v>対応する項目のみ表示</v>
       </c>
       <c r="F7"/>
     </row>
@@ -12516,10 +12476,10 @@
         <v>5</v>
       </c>
       <c r="B8" t="str" s="245">
-        <v>追加部材・オプション</v>
+        <v>室外側の仕上げ・化粧カバー</v>
       </c>
       <c r="C8" t="str" s="245">
-        <v>options</v>
+        <v>exterior_finish</v>
       </c>
       <c r="D8" t="str" s="245">
         <v>選択・確認</v>
@@ -12534,10 +12494,10 @@
         <v>6</v>
       </c>
       <c r="B9" t="str" s="245">
-        <v>選択した部材の仕様</v>
+        <v>追加部材・オプション</v>
       </c>
       <c r="C9" t="str" s="245">
-        <v>part_detail</v>
+        <v>options</v>
       </c>
       <c r="D9" t="str" s="245">
         <v>選択・確認</v>
@@ -12552,33 +12512,53 @@
         <v>7</v>
       </c>
       <c r="B10" t="str" s="245">
-        <v>現場採寸・取付条件</v>
+        <v>選択した部材の仕様</v>
       </c>
       <c r="C10" t="str" s="245">
-        <v>survey</v>
+        <v>part_detail</v>
       </c>
       <c r="D10" t="str" s="245">
         <v>選択・確認</v>
       </c>
       <c r="E10" t="str" s="246">
-        <v>採寸後に再評価</v>
+        <v>対応する項目のみ表示</v>
       </c>
       <c r="F10"/>
     </row>
     <row r="11">
-      <c r="A11" s="244"/>
-      <c r="B11" s="245"/>
-      <c r="C11" s="245"/>
-      <c r="D11" s="245"/>
-      <c r="E11" s="246"/>
+      <c r="A11" t="n" s="244">
+        <v>8</v>
+      </c>
+      <c r="B11" t="str" s="245">
+        <v>現場採寸・取付条件</v>
+      </c>
+      <c r="C11" t="str" s="245">
+        <v>survey</v>
+      </c>
+      <c r="D11" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E11" t="str" s="246">
+        <v>対応する項目のみ表示</v>
+      </c>
       <c r="F11"/>
     </row>
     <row r="12">
-      <c r="A12" s="244"/>
-      <c r="B12" s="245"/>
-      <c r="C12" s="245"/>
-      <c r="D12" s="245"/>
-      <c r="E12" s="246"/>
+      <c r="A12" t="n" s="244">
+        <v>9</v>
+      </c>
+      <c r="B12" t="str" s="245">
+        <v>製品寸法</v>
+      </c>
+      <c r="C12" t="str" s="245">
+        <v>size</v>
+      </c>
+      <c r="D12" t="str" s="245">
+        <v>選択・確認</v>
+      </c>
+      <c r="E12" t="str" s="246">
+        <v>採寸と仕上がりを併記</v>
+      </c>
       <c r="F12"/>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Hide derived Replus confirmation fields while retaining selection dependencies
</commit_message>
<xml_diff>
--- a/changes/replus-runtime-v5/candidates/RPL_ATT_TH.xlsx
+++ b/changes/replus-runtime-v5/candidates/RPL_ATT_TH.xlsx
@@ -1494,7 +1494,7 @@
         <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F3" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="4">
@@ -1514,7 +1514,7 @@
         <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F4" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="5">
@@ -1534,7 +1534,7 @@
         <v>OFFICIAL_SOURCE_REVIEW</v>
       </c>
       <c r="F5" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="6">
@@ -1552,7 +1552,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F6" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="7">
@@ -1572,7 +1572,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F7" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="8">
@@ -1586,13 +1586,13 @@
         <v>new_sash_exterior_color</v>
       </c>
       <c r="D8" t="str" s="245">
-        <v>{"label": "化粧カバー色（外観色に連動）", "group": "exterior_finish", "internal": false}</v>
+        <v>{"label": "化粧カバー色（外観色に連動）", "group": "exterior_finish", "internal": true, "salesDisplay": false}</v>
       </c>
       <c r="E8" t="str" s="246">
-        <v>UI_PRESENTATION</v>
+        <v>USER_PRESENTATION_POLICY</v>
       </c>
       <c r="F8" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="9">
@@ -1606,13 +1606,13 @@
         <v>new_sash_interior_color</v>
       </c>
       <c r="D9" t="str" s="245">
-        <v>{"label": "室内カバー色（内観色に連動）", "group": "interior_finish", "internal": false}</v>
+        <v>{"label": "室内カバー色（内観色に連動）", "group": "interior_finish", "internal": true, "salesDisplay": false}</v>
       </c>
       <c r="E9" t="str" s="246">
-        <v>UI_PRESENTATION</v>
+        <v>USER_PRESENTATION_POLICY</v>
       </c>
       <c r="F9" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="10">
@@ -1632,7 +1632,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F10" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="11">
@@ -1650,7 +1650,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F11" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="12">
@@ -1668,7 +1668,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F12" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="13">
@@ -1686,7 +1686,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F13" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="14">
@@ -1704,7 +1704,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F14" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="15">
@@ -1722,7 +1722,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F15" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="16">
@@ -1740,7 +1740,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F16" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="17">
@@ -1760,7 +1760,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F17" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="18">
@@ -1780,7 +1780,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F18" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="19">
@@ -1800,7 +1800,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F19" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="20">
@@ -1820,7 +1820,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F20" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
     <row r="21">
@@ -1840,7 +1840,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F21" t="str">
-        <v>REPLUS_DIMENSIONS_INNER_FIT_V11_20261014</v>
+        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
       </c>
     </row>
   </sheetData>

</xml_diff>